<commit_message>
Informe semanal 0327 - script Node.js y automatización
</commit_message>
<xml_diff>
--- a/data/informe.xlsx
+++ b/data/informe.xlsx
@@ -5,10 +5,10 @@
   <workbookPr hidePivotFieldList="1"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://everisgroup.sharepoint.com/sites/NTTD-ACNProyectoUP/Documentos compartidos/01. Oficina Técnica/22.Comunicación Informes Consejos/0320/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://everisgroup.sharepoint.com/sites/NTTD-ACNProyectoUP/Documentos compartidos/01. Oficina Técnica/22.Comunicación Informes Consejos/0327/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="125" documentId="8_{CF1B40BF-5534-4499-8EC7-1B1C4491EB18}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{AD1B71DD-3F61-4FE0-9DBF-817DA0E8B955}"/>
+  <xr:revisionPtr revIDLastSave="11" documentId="8_{62AD7D50-223A-4D33-B5F7-4231C7636E2A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E30E5DD9-0680-4A86-AC57-92FBCE0ED73E}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" firstSheet="2" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -24,7 +24,7 @@
   </sheets>
   <calcPr calcId="191029"/>
   <pivotCaches>
-    <pivotCache cacheId="6" r:id="rId9"/>
+    <pivotCache cacheId="0" r:id="rId9"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1290" uniqueCount="406">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1282" uniqueCount="396">
   <si>
     <t>TEMPLATE DE ACTUALIZACIÓN SEMANAL — DASHBOARD FORMACIÓN CONSEJOS</t>
   </si>
@@ -1015,39 +1015,6 @@
     </r>
   </si>
   <si>
-    <t>20/3/2027</t>
-  </si>
-  <si>
-    <t>-La próxima edición de presenciales será en Mallorca el 27 de marzo.</t>
-  </si>
-  <si>
-    <t>-CV de formadores webinar y presenciales.</t>
-  </si>
-  <si>
-    <t>-Quedan pendientes algunas fichas de centro</t>
-  </si>
-  <si>
-    <t xml:space="preserve">-Se espera confirmación de que todas las sesiones de ahora en adelante serán bimodales. </t>
-  </si>
-  <si>
-    <t>-Esperan iniciar los presenciales en junio</t>
-  </si>
-  <si>
-    <t>-Esperan iniciar webinars en mayo</t>
-  </si>
-  <si>
-    <t>-Pendiente la planificación de los webinars</t>
-  </si>
-  <si>
-    <t xml:space="preserve">-Se debe confirmar con el consejo las horas de las sesiones de abril. </t>
-  </si>
-  <si>
-    <t xml:space="preserve"> -Pendiente la planificación de las sesiones presenciales </t>
-  </si>
-  <si>
-    <t>-Las evidencias no se están subiendo correctamente por parte de lso formadores, se debe reforzar la nomenclatura utilizada.</t>
-  </si>
-  <si>
     <t>EP-CGTS-01-A1-ES-014_13032026_1600_Almería</t>
   </si>
   <si>
@@ -1358,6 +1325,9 @@
   </si>
   <si>
     <t>EW-COGITI-02-A5-ES-04EW-COGITI-02-A5-ES-04-003_05032026_1800</t>
+  </si>
+  <si>
+    <t>27/3/2026</t>
   </si>
 </sst>
 </file>
@@ -1573,7 +1543,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="50">
+  <cellXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -1685,6 +1655,15 @@
     <xf numFmtId="14" fontId="4" fillId="9" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="12" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="4" fillId="8" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="4" fillId="8" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1698,16 +1677,6 @@
     <xf numFmtId="0" fontId="8" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="4" fillId="8" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="4" fillId="8" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1926,7 +1895,7 @@
 </file>
 
 <file path=xl/pivotCache/pivotCacheDefinition1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshedBy="Goñi Guarro, Ainhoa" refreshedDate="46100.619546180555" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="414" xr:uid="{0D287A42-7A04-41C6-BB49-5BB5B49D4977}">
+<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshedBy="Goñi Guarro, Ainhoa" refreshedDate="46104.364252893516" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="414" xr:uid="{0D287A42-7A04-41C6-BB49-5BB5B49D4977}">
   <cacheSource type="worksheet">
     <worksheetSource name="Tabla1"/>
   </cacheSource>
@@ -4467,7 +4436,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{4A798B3C-3F81-4257-A53D-F4F2EDDA554E}" name="TablaDinámica1" cacheId="6" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{4A798B3C-3F81-4257-A53D-F4F2EDDA554E}" name="TablaDinámica1" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
   <location ref="A3:K18" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="4">
     <pivotField axis="axisRow" showAll="0" sortType="descending">
@@ -4919,16 +4888,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:3" ht="35.15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B1" s="41" t="s">
+      <c r="B1" s="44" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="42"/>
+      <c r="C1" s="45"/>
     </row>
     <row r="2" spans="2:3" ht="22" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B2" s="43" t="s">
+      <c r="B2" s="46" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="42"/>
+      <c r="C2" s="45"/>
     </row>
     <row r="3" spans="2:3" ht="40" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B3" s="1" t="s">
@@ -5013,10 +4982,10 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:3" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B1" s="44" t="s">
+      <c r="B1" s="47" t="s">
         <v>18</v>
       </c>
-      <c r="C1" s="42"/>
+      <c r="C1" s="45"/>
     </row>
     <row r="2" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B2" s="3" t="s">
@@ -5071,29 +5040,29 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:21" ht="28" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="44" t="s">
+      <c r="A1" s="47" t="s">
         <v>24</v>
       </c>
-      <c r="B1" s="42"/>
-      <c r="C1" s="42"/>
-      <c r="D1" s="42"/>
-      <c r="E1" s="42"/>
-      <c r="F1" s="42"/>
-      <c r="G1" s="42"/>
-      <c r="H1" s="42"/>
-      <c r="I1" s="42"/>
-      <c r="J1" s="42"/>
-      <c r="K1" s="42"/>
-      <c r="L1" s="42"/>
-      <c r="M1" s="42"/>
-      <c r="N1" s="42"/>
-      <c r="O1" s="42"/>
-      <c r="P1" s="42"/>
-      <c r="Q1" s="42"/>
-      <c r="R1" s="42"/>
-      <c r="S1" s="42"/>
-      <c r="T1" s="42"/>
-      <c r="U1" s="42"/>
+      <c r="B1" s="45"/>
+      <c r="C1" s="45"/>
+      <c r="D1" s="45"/>
+      <c r="E1" s="45"/>
+      <c r="F1" s="45"/>
+      <c r="G1" s="45"/>
+      <c r="H1" s="45"/>
+      <c r="I1" s="45"/>
+      <c r="J1" s="45"/>
+      <c r="K1" s="45"/>
+      <c r="L1" s="45"/>
+      <c r="M1" s="45"/>
+      <c r="N1" s="45"/>
+      <c r="O1" s="45"/>
+      <c r="P1" s="45"/>
+      <c r="Q1" s="45"/>
+      <c r="R1" s="45"/>
+      <c r="S1" s="45"/>
+      <c r="T1" s="45"/>
+      <c r="U1" s="45"/>
     </row>
     <row r="2" spans="1:21" ht="26" x14ac:dyDescent="0.35">
       <c r="A2" s="3" t="s">
@@ -5102,7 +5071,7 @@
       <c r="B2" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="C2" s="46" t="s">
+      <c r="C2" s="41" t="s">
         <v>27</v>
       </c>
       <c r="D2" s="3" t="s">
@@ -5164,21 +5133,15 @@
       <c r="A3" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="B3" s="5">
-        <v>719</v>
-      </c>
+      <c r="B3" s="5"/>
       <c r="C3" s="7">
         <v>500</v>
       </c>
       <c r="D3" s="7">
         <v>1250</v>
       </c>
-      <c r="E3" s="18">
-        <v>-8.3000000000000001E-3</v>
-      </c>
-      <c r="F3" s="5">
-        <v>150</v>
-      </c>
+      <c r="E3" s="18"/>
+      <c r="F3" s="5"/>
       <c r="G3" s="7">
         <v>8</v>
       </c>
@@ -5221,21 +5184,15 @@
       <c r="A4" s="6" t="s">
         <v>50</v>
       </c>
-      <c r="B4" s="5">
-        <v>232</v>
-      </c>
+      <c r="B4" s="5"/>
       <c r="C4" s="7">
         <v>140</v>
       </c>
       <c r="D4" s="7">
         <v>350</v>
       </c>
-      <c r="E4" s="18">
-        <v>0</v>
-      </c>
-      <c r="F4" s="5">
-        <v>65</v>
-      </c>
+      <c r="E4" s="18"/>
+      <c r="F4" s="5"/>
       <c r="G4" s="7">
         <v>8</v>
       </c>
@@ -5278,21 +5235,15 @@
       <c r="A5" s="6" t="s">
         <v>52</v>
       </c>
-      <c r="B5" s="13">
-        <v>441</v>
-      </c>
+      <c r="B5" s="13"/>
       <c r="C5" s="7">
         <v>500</v>
       </c>
       <c r="D5" s="7">
         <v>1250</v>
       </c>
-      <c r="E5" s="18">
-        <v>3.7600000000000001E-2</v>
-      </c>
-      <c r="F5" s="5">
-        <v>127</v>
-      </c>
+      <c r="E5" s="18"/>
+      <c r="F5" s="5"/>
       <c r="G5" s="7">
         <v>10</v>
       </c>
@@ -5335,21 +5286,15 @@
       <c r="A6" s="6" t="s">
         <v>54</v>
       </c>
-      <c r="B6" s="5">
-        <v>279</v>
-      </c>
+      <c r="B6" s="5"/>
       <c r="C6" s="7">
         <v>160</v>
       </c>
       <c r="D6" s="7">
         <v>400</v>
       </c>
-      <c r="E6" s="18">
-        <v>-1.41E-2</v>
-      </c>
-      <c r="F6" s="5">
-        <v>4</v>
-      </c>
+      <c r="E6" s="18"/>
+      <c r="F6" s="5"/>
       <c r="G6" s="7">
         <v>10</v>
       </c>
@@ -5392,21 +5337,15 @@
       <c r="A7" s="6" t="s">
         <v>56</v>
       </c>
-      <c r="B7" s="5">
-        <v>231</v>
-      </c>
+      <c r="B7" s="5"/>
       <c r="C7" s="7">
         <v>300</v>
       </c>
       <c r="D7" s="7">
         <v>750</v>
       </c>
-      <c r="E7" s="18">
-        <v>-4.3E-3</v>
-      </c>
-      <c r="F7" s="5">
-        <v>54</v>
-      </c>
+      <c r="E7" s="18"/>
+      <c r="F7" s="5"/>
       <c r="G7" s="7">
         <v>8</v>
       </c>
@@ -5441,33 +5380,23 @@
         <v>4</v>
       </c>
       <c r="R7" s="8"/>
-      <c r="S7" s="21" t="s">
-        <v>298</v>
-      </c>
-      <c r="T7" s="21" t="s">
-        <v>297</v>
-      </c>
+      <c r="S7" s="21"/>
+      <c r="T7" s="21"/>
       <c r="U7" s="8"/>
     </row>
     <row r="8" spans="1:21" ht="60" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A8" s="6" t="s">
         <v>58</v>
       </c>
-      <c r="B8" s="5">
-        <v>1985</v>
-      </c>
+      <c r="B8" s="5"/>
       <c r="C8" s="7">
         <v>1200</v>
       </c>
       <c r="D8" s="7">
         <v>3000</v>
       </c>
-      <c r="E8" s="18">
-        <v>1.6E-2</v>
-      </c>
-      <c r="F8" s="5">
-        <v>434</v>
-      </c>
+      <c r="E8" s="18"/>
+      <c r="F8" s="5"/>
       <c r="G8" s="7">
         <v>9</v>
       </c>
@@ -5501,34 +5430,24 @@
       <c r="Q8" s="5">
         <v>37</v>
       </c>
-      <c r="R8" s="21" t="s">
-        <v>294</v>
-      </c>
+      <c r="R8" s="21"/>
       <c r="S8" s="8"/>
-      <c r="T8" s="21" t="s">
-        <v>293</v>
-      </c>
+      <c r="T8" s="21"/>
       <c r="U8" s="8"/>
     </row>
     <row r="9" spans="1:21" ht="60" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A9" s="6" t="s">
         <v>61</v>
       </c>
-      <c r="B9" s="5">
-        <v>1377</v>
-      </c>
+      <c r="B9" s="5"/>
       <c r="C9" s="7">
         <v>1300</v>
       </c>
       <c r="D9" s="7">
         <v>3250</v>
       </c>
-      <c r="E9" s="19">
-        <v>-2.2000000000000001E-3</v>
-      </c>
-      <c r="F9" s="5">
-        <v>83</v>
-      </c>
+      <c r="E9" s="19"/>
+      <c r="F9" s="5"/>
       <c r="G9" s="7">
         <v>11</v>
       </c>
@@ -5571,21 +5490,15 @@
       <c r="A10" s="6" t="s">
         <v>62</v>
       </c>
-      <c r="B10" s="5">
-        <v>4640</v>
-      </c>
+      <c r="B10" s="5"/>
       <c r="C10" s="7">
         <v>2515</v>
       </c>
       <c r="D10" s="7">
         <v>6287.5</v>
       </c>
-      <c r="E10" s="18">
-        <v>6.0000000000000001E-3</v>
-      </c>
-      <c r="F10" s="5">
-        <v>960</v>
-      </c>
+      <c r="E10" s="18"/>
+      <c r="F10" s="5"/>
       <c r="G10" s="7">
         <v>8</v>
       </c>
@@ -5619,34 +5532,24 @@
       <c r="Q10" s="5">
         <v>0</v>
       </c>
-      <c r="R10" s="21" t="s">
-        <v>295</v>
-      </c>
+      <c r="R10" s="21"/>
       <c r="S10" s="8"/>
-      <c r="T10" s="21" t="s">
-        <v>296</v>
-      </c>
+      <c r="T10" s="21"/>
       <c r="U10" s="8"/>
     </row>
     <row r="11" spans="1:21" ht="60" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A11" s="6" t="s">
         <v>65</v>
       </c>
-      <c r="B11" s="5">
-        <v>23</v>
-      </c>
+      <c r="B11" s="5"/>
       <c r="C11" s="7">
         <v>200</v>
       </c>
       <c r="D11" s="7">
         <v>500</v>
       </c>
-      <c r="E11" s="19">
-        <v>0</v>
-      </c>
-      <c r="F11" s="5">
-        <v>0</v>
-      </c>
+      <c r="E11" s="19"/>
+      <c r="F11" s="5"/>
       <c r="G11" s="7">
         <v>8</v>
       </c>
@@ -5689,21 +5592,15 @@
       <c r="A12" s="6" t="s">
         <v>67</v>
       </c>
-      <c r="B12" s="5">
-        <v>3074</v>
-      </c>
+      <c r="B12" s="5"/>
       <c r="C12" s="7">
         <v>5352</v>
       </c>
       <c r="D12" s="7">
         <v>13380</v>
       </c>
-      <c r="E12" s="18">
-        <v>0.01</v>
-      </c>
-      <c r="F12" s="5">
-        <v>548</v>
-      </c>
+      <c r="E12" s="18"/>
+      <c r="F12" s="5"/>
       <c r="G12" s="7">
         <v>8</v>
       </c>
@@ -5739,30 +5636,22 @@
       </c>
       <c r="R12" s="21"/>
       <c r="S12" s="17"/>
-      <c r="T12" s="21" t="s">
-        <v>301</v>
-      </c>
+      <c r="T12" s="21"/>
       <c r="U12" s="8"/>
     </row>
     <row r="13" spans="1:21" ht="60" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A13" s="6" t="s">
         <v>69</v>
       </c>
-      <c r="B13" s="5">
-        <v>4356</v>
-      </c>
+      <c r="B13" s="5"/>
       <c r="C13" s="7">
         <v>3057</v>
       </c>
       <c r="D13" s="7">
         <v>7642.5</v>
       </c>
-      <c r="E13" s="18">
-        <v>3.0000000000000001E-3</v>
-      </c>
-      <c r="F13" s="5">
-        <v>1132</v>
-      </c>
+      <c r="E13" s="18"/>
+      <c r="F13" s="5"/>
       <c r="G13" s="7">
         <v>10</v>
       </c>
@@ -5805,21 +5694,15 @@
       <c r="A14" s="6" t="s">
         <v>73</v>
       </c>
-      <c r="B14" s="5">
-        <v>426</v>
-      </c>
+      <c r="B14" s="5"/>
       <c r="C14" s="7">
         <v>250</v>
       </c>
       <c r="D14" s="7">
         <v>625</v>
       </c>
-      <c r="E14" s="18">
-        <v>0.01</v>
-      </c>
-      <c r="F14" s="5">
-        <v>60</v>
-      </c>
+      <c r="E14" s="18"/>
+      <c r="F14" s="5"/>
       <c r="G14" s="7">
         <v>8</v>
       </c>
@@ -5862,21 +5745,15 @@
       <c r="A15" s="6" t="s">
         <v>75</v>
       </c>
-      <c r="B15" s="5">
-        <v>336</v>
-      </c>
+      <c r="B15" s="5"/>
       <c r="C15" s="7">
         <v>300</v>
       </c>
       <c r="D15" s="7">
         <v>750</v>
       </c>
-      <c r="E15" s="18">
-        <v>0.11600000000000001</v>
-      </c>
-      <c r="F15" s="5">
-        <v>83</v>
-      </c>
+      <c r="E15" s="18"/>
+      <c r="F15" s="5"/>
       <c r="G15" s="7">
         <v>11</v>
       </c>
@@ -5910,9 +5787,7 @@
       <c r="Q15" s="5">
         <v>12</v>
       </c>
-      <c r="R15" s="21" t="s">
-        <v>300</v>
-      </c>
+      <c r="R15" s="21"/>
       <c r="S15" s="21"/>
       <c r="T15" s="8"/>
       <c r="U15" s="8"/>
@@ -5921,21 +5796,15 @@
       <c r="A16" s="6" t="s">
         <v>79</v>
       </c>
-      <c r="B16" s="5">
-        <v>15059</v>
-      </c>
+      <c r="B16" s="5"/>
       <c r="C16" s="7">
         <v>18664</v>
       </c>
       <c r="D16" s="7">
         <v>46660</v>
       </c>
-      <c r="E16" s="18">
-        <v>4.0000000000000001E-3</v>
-      </c>
-      <c r="F16" s="5">
-        <v>4820</v>
-      </c>
+      <c r="E16" s="18"/>
+      <c r="F16" s="5"/>
       <c r="G16" s="7">
         <v>10</v>
       </c>
@@ -5978,21 +5847,15 @@
       <c r="A17" s="6" t="s">
         <v>80</v>
       </c>
-      <c r="B17" s="5">
-        <v>7385</v>
-      </c>
+      <c r="B17" s="5"/>
       <c r="C17" s="7">
         <v>4014</v>
       </c>
       <c r="D17" s="7">
         <v>10035</v>
       </c>
-      <c r="E17" s="18">
-        <v>1.0999999999999999E-2</v>
-      </c>
-      <c r="F17" s="5">
-        <v>1697</v>
-      </c>
+      <c r="E17" s="18"/>
+      <c r="F17" s="5"/>
       <c r="G17" s="7">
         <v>13</v>
       </c>
@@ -6035,21 +5898,15 @@
       <c r="A18" s="6" t="s">
         <v>82</v>
       </c>
-      <c r="B18" s="5">
-        <v>9274</v>
-      </c>
+      <c r="B18" s="5"/>
       <c r="C18" s="7">
         <v>9300</v>
       </c>
       <c r="D18" s="7">
         <v>23250</v>
       </c>
-      <c r="E18" s="18">
-        <v>5.0000000000000001E-3</v>
-      </c>
-      <c r="F18" s="5">
-        <v>2364</v>
-      </c>
+      <c r="E18" s="18"/>
+      <c r="F18" s="5"/>
       <c r="G18" s="7">
         <v>10</v>
       </c>
@@ -6092,21 +5949,15 @@
       <c r="A19" s="6" t="s">
         <v>85</v>
       </c>
-      <c r="B19" s="5">
-        <v>500</v>
-      </c>
+      <c r="B19" s="5"/>
       <c r="C19" s="7">
         <v>517</v>
       </c>
       <c r="D19" s="7">
         <v>1292.5</v>
       </c>
-      <c r="E19" s="19">
-        <v>2E-3</v>
-      </c>
-      <c r="F19" s="5">
-        <v>14</v>
-      </c>
+      <c r="E19" s="19"/>
+      <c r="F19" s="5"/>
       <c r="G19" s="7">
         <v>8</v>
       </c>
@@ -6149,21 +6000,15 @@
       <c r="A20" s="6" t="s">
         <v>86</v>
       </c>
-      <c r="B20" s="5">
-        <v>309</v>
-      </c>
+      <c r="B20" s="5"/>
       <c r="C20" s="7">
         <v>215</v>
       </c>
       <c r="D20" s="7">
         <v>537.5</v>
       </c>
-      <c r="E20" s="18">
-        <v>0</v>
-      </c>
-      <c r="F20" s="5">
-        <v>117</v>
-      </c>
+      <c r="E20" s="18"/>
+      <c r="F20" s="5"/>
       <c r="G20" s="7">
         <v>8</v>
       </c>
@@ -6198,9 +6043,7 @@
         <v>0</v>
       </c>
       <c r="R20" s="8"/>
-      <c r="S20" s="21" t="s">
-        <v>299</v>
-      </c>
+      <c r="S20" s="21"/>
       <c r="T20" s="8"/>
       <c r="U20" s="8"/>
     </row>
@@ -6208,21 +6051,15 @@
       <c r="A21" s="6" t="s">
         <v>89</v>
       </c>
-      <c r="B21" s="5">
-        <v>23179</v>
-      </c>
+      <c r="B21" s="5"/>
       <c r="C21" s="7">
         <v>31516</v>
       </c>
       <c r="D21" s="7">
         <v>78790</v>
       </c>
-      <c r="E21" s="18">
-        <v>1.24E-2</v>
-      </c>
-      <c r="F21" s="5">
-        <v>9989</v>
-      </c>
+      <c r="E21" s="18"/>
+      <c r="F21" s="5"/>
       <c r="G21" s="7">
         <v>12</v>
       </c>
@@ -6256,9 +6093,7 @@
       <c r="Q21" s="5">
         <v>11</v>
       </c>
-      <c r="R21" s="21" t="s">
-        <v>302</v>
-      </c>
+      <c r="R21" s="21"/>
       <c r="S21" s="8"/>
       <c r="T21" s="21"/>
       <c r="U21" s="21"/>
@@ -6337,22 +6172,16 @@
       <c r="A5" s="29" t="s">
         <v>82</v>
       </c>
-      <c r="B5" s="49"/>
-      <c r="C5" s="49">
+      <c r="C5">
         <v>6</v>
       </c>
-      <c r="D5" s="49">
+      <c r="D5">
         <v>41</v>
       </c>
-      <c r="E5" s="49"/>
-      <c r="F5" s="49">
+      <c r="F5">
         <v>37</v>
       </c>
-      <c r="G5" s="49"/>
-      <c r="H5" s="49"/>
-      <c r="I5" s="49"/>
-      <c r="J5" s="49"/>
-      <c r="K5" s="49">
+      <c r="K5">
         <v>84</v>
       </c>
     </row>
@@ -6360,26 +6189,22 @@
       <c r="A6" s="29" t="s">
         <v>62</v>
       </c>
-      <c r="B6" s="49">
+      <c r="B6">
         <v>4</v>
       </c>
-      <c r="C6" s="49">
+      <c r="C6">
         <v>19</v>
       </c>
-      <c r="D6" s="49">
+      <c r="D6">
         <v>20</v>
       </c>
-      <c r="E6" s="49"/>
-      <c r="F6" s="49">
+      <c r="F6">
         <v>21</v>
       </c>
-      <c r="G6" s="49"/>
-      <c r="H6" s="49">
+      <c r="H6">
         <v>3</v>
       </c>
-      <c r="I6" s="49"/>
-      <c r="J6" s="49"/>
-      <c r="K6" s="49">
+      <c r="K6">
         <v>67</v>
       </c>
     </row>
@@ -6387,24 +6212,19 @@
       <c r="A7" s="29" t="s">
         <v>61</v>
       </c>
-      <c r="B7" s="49"/>
-      <c r="C7" s="49"/>
-      <c r="D7" s="49">
+      <c r="D7">
         <v>20</v>
       </c>
-      <c r="E7" s="49"/>
-      <c r="F7" s="49">
+      <c r="F7">
         <v>40</v>
       </c>
-      <c r="G7" s="49">
+      <c r="G7">
         <v>3</v>
       </c>
-      <c r="H7" s="49">
+      <c r="H7">
         <v>4</v>
       </c>
-      <c r="I7" s="49"/>
-      <c r="J7" s="49"/>
-      <c r="K7" s="49">
+      <c r="K7">
         <v>67</v>
       </c>
     </row>
@@ -6412,28 +6232,25 @@
       <c r="A8" s="29" t="s">
         <v>89</v>
       </c>
-      <c r="B8" s="49">
+      <c r="B8">
         <v>14</v>
       </c>
-      <c r="C8" s="49">
+      <c r="C8">
         <v>15</v>
       </c>
-      <c r="D8" s="49">
+      <c r="D8">
         <v>5</v>
       </c>
-      <c r="E8" s="49"/>
-      <c r="F8" s="49">
+      <c r="F8">
         <v>8</v>
       </c>
-      <c r="G8" s="49">
+      <c r="G8">
         <v>1</v>
       </c>
-      <c r="H8" s="49">
+      <c r="H8">
         <v>8</v>
       </c>
-      <c r="I8" s="49"/>
-      <c r="J8" s="49"/>
-      <c r="K8" s="49">
+      <c r="K8">
         <v>51</v>
       </c>
     </row>
@@ -6441,26 +6258,22 @@
       <c r="A9" s="29" t="s">
         <v>58</v>
       </c>
-      <c r="B9" s="49">
+      <c r="B9">
         <v>4</v>
       </c>
-      <c r="C9" s="49">
+      <c r="C9">
         <v>4</v>
       </c>
-      <c r="D9" s="49">
+      <c r="D9">
         <v>2</v>
       </c>
-      <c r="E9" s="49"/>
-      <c r="F9" s="49"/>
-      <c r="G9" s="49"/>
-      <c r="H9" s="49">
+      <c r="H9">
         <v>4</v>
       </c>
-      <c r="I9" s="49">
+      <c r="I9">
         <v>16</v>
       </c>
-      <c r="J9" s="49"/>
-      <c r="K9" s="49">
+      <c r="K9">
         <v>30</v>
       </c>
     </row>
@@ -6468,24 +6281,19 @@
       <c r="A10" s="29" t="s">
         <v>75</v>
       </c>
-      <c r="B10" s="49"/>
-      <c r="C10" s="49"/>
-      <c r="D10" s="49">
+      <c r="D10">
         <v>4</v>
       </c>
-      <c r="E10" s="49"/>
-      <c r="F10" s="49">
+      <c r="F10">
         <v>8</v>
       </c>
-      <c r="G10" s="49">
+      <c r="G10">
         <v>4</v>
       </c>
-      <c r="H10" s="49">
+      <c r="H10">
         <v>4</v>
       </c>
-      <c r="I10" s="49"/>
-      <c r="J10" s="49"/>
-      <c r="K10" s="49">
+      <c r="K10">
         <v>20</v>
       </c>
     </row>
@@ -6493,18 +6301,10 @@
       <c r="A11" s="29" t="s">
         <v>79</v>
       </c>
-      <c r="B11" s="49"/>
-      <c r="C11" s="49"/>
-      <c r="D11" s="49"/>
-      <c r="E11" s="49"/>
-      <c r="F11" s="49"/>
-      <c r="G11" s="49"/>
-      <c r="H11" s="49">
+      <c r="H11">
         <v>8</v>
       </c>
-      <c r="I11" s="49"/>
-      <c r="J11" s="49"/>
-      <c r="K11" s="49">
+      <c r="K11">
         <v>8</v>
       </c>
     </row>
@@ -6512,22 +6312,16 @@
       <c r="A12" s="29" t="s">
         <v>67</v>
       </c>
-      <c r="B12" s="49"/>
-      <c r="C12" s="49"/>
-      <c r="D12" s="49"/>
-      <c r="E12" s="49"/>
-      <c r="F12" s="49"/>
-      <c r="G12" s="49">
+      <c r="G12">
         <v>3</v>
       </c>
-      <c r="H12" s="49">
+      <c r="H12">
         <v>3</v>
       </c>
-      <c r="I12" s="49">
+      <c r="I12">
         <v>1</v>
       </c>
-      <c r="J12" s="49"/>
-      <c r="K12" s="49">
+      <c r="K12">
         <v>7</v>
       </c>
     </row>
@@ -6535,22 +6329,16 @@
       <c r="A13" s="29" t="s">
         <v>85</v>
       </c>
-      <c r="B13" s="49"/>
-      <c r="C13" s="49"/>
-      <c r="D13" s="49">
+      <c r="D13">
         <v>1</v>
       </c>
-      <c r="E13" s="49"/>
-      <c r="F13" s="49">
+      <c r="F13">
         <v>2</v>
       </c>
-      <c r="G13" s="49">
+      <c r="G13">
         <v>1</v>
       </c>
-      <c r="H13" s="49"/>
-      <c r="I13" s="49"/>
-      <c r="J13" s="49"/>
-      <c r="K13" s="49">
+      <c r="K13">
         <v>4</v>
       </c>
     </row>
@@ -6558,20 +6346,13 @@
       <c r="A14" s="29" t="s">
         <v>69</v>
       </c>
-      <c r="B14" s="49"/>
-      <c r="C14" s="49"/>
-      <c r="D14" s="49">
+      <c r="D14">
         <v>1</v>
       </c>
-      <c r="E14" s="49"/>
-      <c r="F14" s="49"/>
-      <c r="G14" s="49"/>
-      <c r="H14" s="49">
+      <c r="H14">
         <v>1</v>
       </c>
-      <c r="I14" s="49"/>
-      <c r="J14" s="49"/>
-      <c r="K14" s="49">
+      <c r="K14">
         <v>2</v>
       </c>
     </row>
@@ -6579,20 +6360,13 @@
       <c r="A15" s="29" t="s">
         <v>73</v>
       </c>
-      <c r="B15" s="49"/>
-      <c r="C15" s="49"/>
-      <c r="D15" s="49"/>
-      <c r="E15" s="49">
+      <c r="E15">
         <v>1</v>
       </c>
-      <c r="F15" s="49"/>
-      <c r="G15" s="49"/>
-      <c r="H15" s="49"/>
-      <c r="I15" s="49">
+      <c r="I15">
         <v>1</v>
       </c>
-      <c r="J15" s="49"/>
-      <c r="K15" s="49">
+      <c r="K15">
         <v>2</v>
       </c>
     </row>
@@ -6600,20 +6374,13 @@
       <c r="A16" s="29" t="s">
         <v>46</v>
       </c>
-      <c r="B16" s="49"/>
-      <c r="C16" s="49"/>
-      <c r="D16" s="49"/>
-      <c r="E16" s="49"/>
-      <c r="F16" s="49"/>
-      <c r="G16" s="49">
+      <c r="G16">
         <v>1</v>
       </c>
-      <c r="H16" s="49">
+      <c r="H16">
         <v>1</v>
       </c>
-      <c r="I16" s="49"/>
-      <c r="J16" s="49"/>
-      <c r="K16" s="49">
+      <c r="K16">
         <v>2</v>
       </c>
     </row>
@@ -6621,47 +6388,36 @@
       <c r="A17" s="29" t="s">
         <v>284</v>
       </c>
-      <c r="B17" s="49"/>
-      <c r="C17" s="49"/>
-      <c r="D17" s="49"/>
-      <c r="E17" s="49"/>
-      <c r="F17" s="49"/>
-      <c r="G17" s="49"/>
-      <c r="H17" s="49"/>
-      <c r="I17" s="49"/>
-      <c r="J17" s="49"/>
-      <c r="K17" s="49"/>
     </row>
     <row r="18" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A18" s="29" t="s">
         <v>285</v>
       </c>
-      <c r="B18" s="49">
+      <c r="B18">
         <v>22</v>
       </c>
-      <c r="C18" s="49">
+      <c r="C18">
         <v>44</v>
       </c>
-      <c r="D18" s="49">
+      <c r="D18">
         <v>94</v>
       </c>
-      <c r="E18" s="49">
+      <c r="E18">
         <v>1</v>
       </c>
-      <c r="F18" s="49">
+      <c r="F18">
         <v>116</v>
       </c>
-      <c r="G18" s="49">
+      <c r="G18">
         <v>13</v>
       </c>
-      <c r="H18" s="49">
+      <c r="H18">
         <v>36</v>
       </c>
-      <c r="I18" s="49">
+      <c r="I18">
         <v>18</v>
       </c>
-      <c r="J18" s="49"/>
-      <c r="K18" s="49">
+      <c r="K18">
         <v>344</v>
       </c>
     </row>
@@ -6682,12 +6438,12 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="28" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="44" t="s">
+      <c r="A1" s="47" t="s">
         <v>91</v>
       </c>
-      <c r="B1" s="42"/>
-      <c r="C1" s="42"/>
-      <c r="D1" s="42"/>
+      <c r="B1" s="45"/>
+      <c r="C1" s="45"/>
+      <c r="D1" s="45"/>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A2" s="32" t="s">
@@ -7944,7 +7700,7 @@
         <v>62</v>
       </c>
       <c r="B106" s="33" t="s">
-        <v>303</v>
+        <v>292</v>
       </c>
       <c r="C106" s="36" t="s">
         <v>133</v>
@@ -7956,7 +7712,7 @@
         <v>62</v>
       </c>
       <c r="B107" s="33" t="s">
-        <v>303</v>
+        <v>292</v>
       </c>
       <c r="C107" s="36" t="s">
         <v>134</v>
@@ -7968,7 +7724,7 @@
         <v>62</v>
       </c>
       <c r="B108" s="33" t="s">
-        <v>304</v>
+        <v>293</v>
       </c>
       <c r="C108" s="36" t="s">
         <v>133</v>
@@ -7980,7 +7736,7 @@
         <v>62</v>
       </c>
       <c r="B109" s="33" t="s">
-        <v>304</v>
+        <v>293</v>
       </c>
       <c r="C109" s="36" t="s">
         <v>134</v>
@@ -7992,7 +7748,7 @@
         <v>62</v>
       </c>
       <c r="B110" s="33" t="s">
-        <v>305</v>
+        <v>294</v>
       </c>
       <c r="C110" s="36" t="s">
         <v>133</v>
@@ -8004,7 +7760,7 @@
         <v>62</v>
       </c>
       <c r="B111" s="33" t="s">
-        <v>305</v>
+        <v>294</v>
       </c>
       <c r="C111" s="36" t="s">
         <v>134</v>
@@ -8016,7 +7772,7 @@
         <v>62</v>
       </c>
       <c r="B112" s="33" t="s">
-        <v>306</v>
+        <v>295</v>
       </c>
       <c r="C112" s="36" t="s">
         <v>132</v>
@@ -8028,7 +7784,7 @@
         <v>62</v>
       </c>
       <c r="B113" s="33" t="s">
-        <v>306</v>
+        <v>295</v>
       </c>
       <c r="C113" s="36" t="s">
         <v>133</v>
@@ -8040,7 +7796,7 @@
         <v>62</v>
       </c>
       <c r="B114" s="33" t="s">
-        <v>306</v>
+        <v>295</v>
       </c>
       <c r="C114" s="36" t="s">
         <v>134</v>
@@ -8052,7 +7808,7 @@
         <v>62</v>
       </c>
       <c r="B115" s="33" t="s">
-        <v>307</v>
+        <v>296</v>
       </c>
       <c r="C115" s="36" t="s">
         <v>132</v>
@@ -8064,7 +7820,7 @@
         <v>62</v>
       </c>
       <c r="B116" s="33" t="s">
-        <v>307</v>
+        <v>296</v>
       </c>
       <c r="C116" s="36" t="s">
         <v>133</v>
@@ -8076,7 +7832,7 @@
         <v>62</v>
       </c>
       <c r="B117" s="33" t="s">
-        <v>307</v>
+        <v>296</v>
       </c>
       <c r="C117" s="36" t="s">
         <v>134</v>
@@ -8088,7 +7844,7 @@
         <v>62</v>
       </c>
       <c r="B118" s="33" t="s">
-        <v>308</v>
+        <v>297</v>
       </c>
       <c r="C118" s="36" t="s">
         <v>132</v>
@@ -8100,7 +7856,7 @@
         <v>62</v>
       </c>
       <c r="B119" s="33" t="s">
-        <v>308</v>
+        <v>297</v>
       </c>
       <c r="C119" s="36" t="s">
         <v>133</v>
@@ -8112,7 +7868,7 @@
         <v>62</v>
       </c>
       <c r="B120" s="33" t="s">
-        <v>308</v>
+        <v>297</v>
       </c>
       <c r="C120" s="36" t="s">
         <v>134</v>
@@ -8196,7 +7952,7 @@
         <v>89</v>
       </c>
       <c r="B127" s="33" t="s">
-        <v>309</v>
+        <v>298</v>
       </c>
       <c r="C127" s="36" t="s">
         <v>133</v>
@@ -8208,7 +7964,7 @@
         <v>89</v>
       </c>
       <c r="B128" s="33" t="s">
-        <v>309</v>
+        <v>298</v>
       </c>
       <c r="C128" s="36" t="s">
         <v>134</v>
@@ -8292,7 +8048,7 @@
         <v>89</v>
       </c>
       <c r="B135" s="33" t="s">
-        <v>310</v>
+        <v>299</v>
       </c>
       <c r="C135" s="36" t="s">
         <v>131</v>
@@ -8304,7 +8060,7 @@
         <v>89</v>
       </c>
       <c r="B136" s="33" t="s">
-        <v>310</v>
+        <v>299</v>
       </c>
       <c r="C136" s="36" t="s">
         <v>132</v>
@@ -8316,7 +8072,7 @@
         <v>89</v>
       </c>
       <c r="B137" s="33" t="s">
-        <v>310</v>
+        <v>299</v>
       </c>
       <c r="C137" s="36" t="s">
         <v>134</v>
@@ -8448,7 +8204,7 @@
         <v>89</v>
       </c>
       <c r="B148" s="33" t="s">
-        <v>311</v>
+        <v>300</v>
       </c>
       <c r="C148" s="36" t="s">
         <v>131</v>
@@ -8460,7 +8216,7 @@
         <v>89</v>
       </c>
       <c r="B149" s="33" t="s">
-        <v>311</v>
+        <v>300</v>
       </c>
       <c r="C149" s="36" t="s">
         <v>132</v>
@@ -8472,7 +8228,7 @@
         <v>89</v>
       </c>
       <c r="B150" s="33" t="s">
-        <v>312</v>
+        <v>301</v>
       </c>
       <c r="C150" s="36" t="s">
         <v>131</v>
@@ -8484,7 +8240,7 @@
         <v>89</v>
       </c>
       <c r="B151" s="33" t="s">
-        <v>312</v>
+        <v>301</v>
       </c>
       <c r="C151" s="36" t="s">
         <v>132</v>
@@ -8496,7 +8252,7 @@
         <v>89</v>
       </c>
       <c r="B152" s="33" t="s">
-        <v>313</v>
+        <v>302</v>
       </c>
       <c r="C152" s="36" t="s">
         <v>131</v>
@@ -8508,7 +8264,7 @@
         <v>89</v>
       </c>
       <c r="B153" s="33" t="s">
-        <v>313</v>
+        <v>302</v>
       </c>
       <c r="C153" s="36" t="s">
         <v>132</v>
@@ -8520,7 +8276,7 @@
         <v>89</v>
       </c>
       <c r="B154" s="33" t="s">
-        <v>313</v>
+        <v>302</v>
       </c>
       <c r="C154" s="36" t="s">
         <v>134</v>
@@ -8532,7 +8288,7 @@
         <v>89</v>
       </c>
       <c r="B155" s="33" t="s">
-        <v>314</v>
+        <v>303</v>
       </c>
       <c r="C155" s="36" t="s">
         <v>131</v>
@@ -8544,7 +8300,7 @@
         <v>89</v>
       </c>
       <c r="B156" s="33" t="s">
-        <v>314</v>
+        <v>303</v>
       </c>
       <c r="C156" s="36" t="s">
         <v>132</v>
@@ -8556,7 +8312,7 @@
         <v>89</v>
       </c>
       <c r="B157" s="33" t="s">
-        <v>314</v>
+        <v>303</v>
       </c>
       <c r="C157" s="36" t="s">
         <v>134</v>
@@ -8568,7 +8324,7 @@
         <v>89</v>
       </c>
       <c r="B158" s="33" t="s">
-        <v>315</v>
+        <v>304</v>
       </c>
       <c r="C158" s="36" t="s">
         <v>131</v>
@@ -8580,7 +8336,7 @@
         <v>89</v>
       </c>
       <c r="B159" s="33" t="s">
-        <v>315</v>
+        <v>304</v>
       </c>
       <c r="C159" s="36" t="s">
         <v>132</v>
@@ -8592,7 +8348,7 @@
         <v>89</v>
       </c>
       <c r="B160" s="33" t="s">
-        <v>315</v>
+        <v>304</v>
       </c>
       <c r="C160" s="36" t="s">
         <v>134</v>
@@ -8604,7 +8360,7 @@
         <v>89</v>
       </c>
       <c r="B161" s="33" t="s">
-        <v>316</v>
+        <v>305</v>
       </c>
       <c r="C161" s="36" t="s">
         <v>131</v>
@@ -8616,7 +8372,7 @@
         <v>89</v>
       </c>
       <c r="B162" s="33" t="s">
-        <v>316</v>
+        <v>305</v>
       </c>
       <c r="C162" s="36" t="s">
         <v>132</v>
@@ -8628,7 +8384,7 @@
         <v>89</v>
       </c>
       <c r="B163" s="33" t="s">
-        <v>316</v>
+        <v>305</v>
       </c>
       <c r="C163" s="36" t="s">
         <v>131</v>
@@ -8640,7 +8396,7 @@
         <v>89</v>
       </c>
       <c r="B164" s="33" t="s">
-        <v>316</v>
+        <v>305</v>
       </c>
       <c r="C164" s="36" t="s">
         <v>132</v>
@@ -8652,7 +8408,7 @@
         <v>89</v>
       </c>
       <c r="B165" s="33" t="s">
-        <v>316</v>
+        <v>305</v>
       </c>
       <c r="C165" s="36" t="s">
         <v>131</v>
@@ -8664,7 +8420,7 @@
         <v>89</v>
       </c>
       <c r="B166" s="33" t="s">
-        <v>316</v>
+        <v>305</v>
       </c>
       <c r="C166" s="36" t="s">
         <v>132</v>
@@ -8676,7 +8432,7 @@
         <v>89</v>
       </c>
       <c r="B167" s="33" t="s">
-        <v>316</v>
+        <v>305</v>
       </c>
       <c r="C167" s="36" t="s">
         <v>131</v>
@@ -8688,7 +8444,7 @@
         <v>89</v>
       </c>
       <c r="B168" s="33" t="s">
-        <v>316</v>
+        <v>305</v>
       </c>
       <c r="C168" s="36" t="s">
         <v>132</v>
@@ -8820,7 +8576,7 @@
         <v>75</v>
       </c>
       <c r="B179" s="33" t="s">
-        <v>317</v>
+        <v>306</v>
       </c>
       <c r="C179" s="36" t="s">
         <v>133</v>
@@ -8832,7 +8588,7 @@
         <v>75</v>
       </c>
       <c r="B180" s="33" t="s">
-        <v>317</v>
+        <v>306</v>
       </c>
       <c r="C180" s="36" t="s">
         <v>134</v>
@@ -8916,7 +8672,7 @@
         <v>58</v>
       </c>
       <c r="B187" s="33" t="s">
-        <v>318</v>
+        <v>307</v>
       </c>
       <c r="C187" s="36" t="s">
         <v>131</v>
@@ -8928,7 +8684,7 @@
         <v>58</v>
       </c>
       <c r="B188" s="33" t="s">
-        <v>318</v>
+        <v>307</v>
       </c>
       <c r="C188" s="36" t="s">
         <v>132</v>
@@ -8940,7 +8696,7 @@
         <v>58</v>
       </c>
       <c r="B189" s="33" t="s">
-        <v>319</v>
+        <v>308</v>
       </c>
       <c r="C189" s="36" t="s">
         <v>131</v>
@@ -8952,7 +8708,7 @@
         <v>58</v>
       </c>
       <c r="B190" s="33" t="s">
-        <v>319</v>
+        <v>308</v>
       </c>
       <c r="C190" s="36" t="s">
         <v>132</v>
@@ -8964,7 +8720,7 @@
         <v>69</v>
       </c>
       <c r="B191" s="33" t="s">
-        <v>320</v>
+        <v>309</v>
       </c>
       <c r="C191" s="36" t="s">
         <v>133</v>
@@ -8976,7 +8732,7 @@
         <v>85</v>
       </c>
       <c r="B192" s="33" t="s">
-        <v>321</v>
+        <v>310</v>
       </c>
       <c r="C192" s="36" t="s">
         <v>133</v>
@@ -8988,7 +8744,7 @@
         <v>85</v>
       </c>
       <c r="B193" s="33" t="s">
-        <v>322</v>
+        <v>311</v>
       </c>
       <c r="C193" s="36" t="s">
         <v>134</v>
@@ -9000,7 +8756,7 @@
         <v>85</v>
       </c>
       <c r="B194" s="33" t="s">
-        <v>323</v>
+        <v>312</v>
       </c>
       <c r="C194" s="36" t="s">
         <v>134</v>
@@ -9180,7 +8936,7 @@
         <v>82</v>
       </c>
       <c r="B209" s="33" t="s">
-        <v>324</v>
+        <v>313</v>
       </c>
       <c r="C209" s="36" t="s">
         <v>134</v>
@@ -9192,7 +8948,7 @@
         <v>82</v>
       </c>
       <c r="B210" s="33" t="s">
-        <v>325</v>
+        <v>314</v>
       </c>
       <c r="C210" s="36" t="s">
         <v>134</v>
@@ -9204,7 +8960,7 @@
         <v>82</v>
       </c>
       <c r="B211" s="33" t="s">
-        <v>326</v>
+        <v>315</v>
       </c>
       <c r="C211" s="36" t="s">
         <v>134</v>
@@ -9216,7 +8972,7 @@
         <v>82</v>
       </c>
       <c r="B212" s="33" t="s">
-        <v>327</v>
+        <v>316</v>
       </c>
       <c r="C212" s="36" t="s">
         <v>133</v>
@@ -9228,7 +8984,7 @@
         <v>82</v>
       </c>
       <c r="B213" s="33" t="s">
-        <v>328</v>
+        <v>317</v>
       </c>
       <c r="C213" s="36" t="s">
         <v>133</v>
@@ -9240,7 +8996,7 @@
         <v>82</v>
       </c>
       <c r="B214" s="33" t="s">
-        <v>329</v>
+        <v>318</v>
       </c>
       <c r="C214" s="36" t="s">
         <v>133</v>
@@ -9312,7 +9068,7 @@
         <v>82</v>
       </c>
       <c r="B220" s="33" t="s">
-        <v>330</v>
+        <v>319</v>
       </c>
       <c r="C220" s="36" t="s">
         <v>134</v>
@@ -9336,7 +9092,7 @@
         <v>82</v>
       </c>
       <c r="B222" s="33" t="s">
-        <v>331</v>
+        <v>320</v>
       </c>
       <c r="C222" s="36" t="s">
         <v>133</v>
@@ -9348,7 +9104,7 @@
         <v>82</v>
       </c>
       <c r="B223" s="33" t="s">
-        <v>332</v>
+        <v>321</v>
       </c>
       <c r="C223" s="36" t="s">
         <v>133</v>
@@ -9360,7 +9116,7 @@
         <v>82</v>
       </c>
       <c r="B224" s="33" t="s">
-        <v>332</v>
+        <v>321</v>
       </c>
       <c r="C224" s="36" t="s">
         <v>134</v>
@@ -9396,7 +9152,7 @@
         <v>82</v>
       </c>
       <c r="B227" s="33" t="s">
-        <v>333</v>
+        <v>322</v>
       </c>
       <c r="C227" s="36" t="s">
         <v>133</v>
@@ -9468,7 +9224,7 @@
         <v>82</v>
       </c>
       <c r="B233" s="33" t="s">
-        <v>334</v>
+        <v>323</v>
       </c>
       <c r="C233" s="36" t="s">
         <v>134</v>
@@ -9480,7 +9236,7 @@
         <v>82</v>
       </c>
       <c r="B234" s="33" t="s">
-        <v>335</v>
+        <v>324</v>
       </c>
       <c r="C234" s="36" t="s">
         <v>134</v>
@@ -9504,7 +9260,7 @@
         <v>82</v>
       </c>
       <c r="B236" s="33" t="s">
-        <v>336</v>
+        <v>325</v>
       </c>
       <c r="C236" s="36" t="s">
         <v>134</v>
@@ -9516,7 +9272,7 @@
         <v>82</v>
       </c>
       <c r="B237" s="33" t="s">
-        <v>337</v>
+        <v>326</v>
       </c>
       <c r="C237" s="36" t="s">
         <v>134</v>
@@ -9576,7 +9332,7 @@
         <v>82</v>
       </c>
       <c r="B242" s="33" t="s">
-        <v>338</v>
+        <v>327</v>
       </c>
       <c r="C242" s="36" t="s">
         <v>134</v>
@@ -9600,7 +9356,7 @@
         <v>82</v>
       </c>
       <c r="B244" s="33" t="s">
-        <v>339</v>
+        <v>328</v>
       </c>
       <c r="C244" s="36" t="s">
         <v>134</v>
@@ -9696,7 +9452,7 @@
         <v>82</v>
       </c>
       <c r="B252" s="33" t="s">
-        <v>340</v>
+        <v>329</v>
       </c>
       <c r="C252" s="36" t="s">
         <v>134</v>
@@ -9708,7 +9464,7 @@
         <v>82</v>
       </c>
       <c r="B253" s="33" t="s">
-        <v>341</v>
+        <v>330</v>
       </c>
       <c r="C253" s="36" t="s">
         <v>134</v>
@@ -9768,7 +9524,7 @@
         <v>82</v>
       </c>
       <c r="B258" s="31" t="s">
-        <v>342</v>
+        <v>331</v>
       </c>
       <c r="C258" s="37" t="s">
         <v>133</v>
@@ -9816,7 +9572,7 @@
         <v>82</v>
       </c>
       <c r="B262" s="31" t="s">
-        <v>343</v>
+        <v>332</v>
       </c>
       <c r="C262" s="37" t="s">
         <v>133</v>
@@ -9828,7 +9584,7 @@
         <v>82</v>
       </c>
       <c r="B263" s="31" t="s">
-        <v>344</v>
+        <v>333</v>
       </c>
       <c r="C263" s="37" t="s">
         <v>134</v>
@@ -9840,7 +9596,7 @@
         <v>82</v>
       </c>
       <c r="B264" s="31" t="s">
-        <v>345</v>
+        <v>334</v>
       </c>
       <c r="C264" s="37" t="s">
         <v>134</v>
@@ -9852,7 +9608,7 @@
         <v>82</v>
       </c>
       <c r="B265" s="31" t="s">
-        <v>346</v>
+        <v>335</v>
       </c>
       <c r="C265" s="37" t="s">
         <v>134</v>
@@ -9864,7 +9620,7 @@
         <v>82</v>
       </c>
       <c r="B266" s="31" t="s">
-        <v>347</v>
+        <v>336</v>
       </c>
       <c r="C266" s="37" t="s">
         <v>134</v>
@@ -9936,7 +9692,7 @@
         <v>82</v>
       </c>
       <c r="B272" s="31" t="s">
-        <v>348</v>
+        <v>337</v>
       </c>
       <c r="C272" s="37" t="s">
         <v>133</v>
@@ -9948,7 +9704,7 @@
         <v>82</v>
       </c>
       <c r="B273" s="31" t="s">
-        <v>349</v>
+        <v>338</v>
       </c>
       <c r="C273" s="37" t="s">
         <v>133</v>
@@ -9960,7 +9716,7 @@
         <v>82</v>
       </c>
       <c r="B274" s="31" t="s">
-        <v>350</v>
+        <v>339</v>
       </c>
       <c r="C274" s="37" t="s">
         <v>133</v>
@@ -9972,7 +9728,7 @@
         <v>82</v>
       </c>
       <c r="B275" s="31" t="s">
-        <v>351</v>
+        <v>340</v>
       </c>
       <c r="C275" s="37" t="s">
         <v>133</v>
@@ -9984,7 +9740,7 @@
         <v>82</v>
       </c>
       <c r="B276" s="31" t="s">
-        <v>352</v>
+        <v>341</v>
       </c>
       <c r="C276" s="37" t="s">
         <v>133</v>
@@ -9996,7 +9752,7 @@
         <v>82</v>
       </c>
       <c r="B277" s="31" t="s">
-        <v>353</v>
+        <v>342</v>
       </c>
       <c r="C277" s="37" t="s">
         <v>132</v>
@@ -10008,7 +9764,7 @@
         <v>82</v>
       </c>
       <c r="B278" s="31" t="s">
-        <v>354</v>
+        <v>343</v>
       </c>
       <c r="C278" s="37" t="s">
         <v>132</v>
@@ -10068,7 +9824,7 @@
         <v>89</v>
       </c>
       <c r="B283" s="31" t="s">
-        <v>355</v>
+        <v>344</v>
       </c>
       <c r="C283" s="37" t="s">
         <v>138</v>
@@ -10080,7 +9836,7 @@
         <v>89</v>
       </c>
       <c r="B284" s="31" t="s">
-        <v>356</v>
+        <v>345</v>
       </c>
       <c r="C284" s="37" t="s">
         <v>138</v>
@@ -10092,7 +9848,7 @@
         <v>89</v>
       </c>
       <c r="B285" s="31" t="s">
-        <v>357</v>
+        <v>346</v>
       </c>
       <c r="C285" s="37" t="s">
         <v>138</v>
@@ -10104,7 +9860,7 @@
         <v>89</v>
       </c>
       <c r="B286" s="31" t="s">
-        <v>357</v>
+        <v>346</v>
       </c>
       <c r="C286" s="37" t="s">
         <v>235</v>
@@ -10116,7 +9872,7 @@
         <v>89</v>
       </c>
       <c r="B287" s="31" t="s">
-        <v>358</v>
+        <v>347</v>
       </c>
       <c r="C287" s="37" t="s">
         <v>138</v>
@@ -10128,7 +9884,7 @@
         <v>61</v>
       </c>
       <c r="B288" s="31" t="s">
-        <v>359</v>
+        <v>348</v>
       </c>
       <c r="C288" s="37" t="s">
         <v>138</v>
@@ -10140,7 +9896,7 @@
         <v>61</v>
       </c>
       <c r="B289" s="31" t="s">
-        <v>360</v>
+        <v>349</v>
       </c>
       <c r="C289" s="37" t="s">
         <v>138</v>
@@ -10152,7 +9908,7 @@
         <v>61</v>
       </c>
       <c r="B290" s="31" t="s">
-        <v>361</v>
+        <v>350</v>
       </c>
       <c r="C290" s="37" t="s">
         <v>235</v>
@@ -10164,7 +9920,7 @@
         <v>61</v>
       </c>
       <c r="B291" s="31" t="s">
-        <v>362</v>
+        <v>351</v>
       </c>
       <c r="C291" s="37" t="s">
         <v>235</v>
@@ -10176,7 +9932,7 @@
         <v>61</v>
       </c>
       <c r="B292" s="31" t="s">
-        <v>363</v>
+        <v>352</v>
       </c>
       <c r="C292" s="37" t="s">
         <v>235</v>
@@ -10188,7 +9944,7 @@
         <v>61</v>
       </c>
       <c r="B293" s="31" t="s">
-        <v>364</v>
+        <v>353</v>
       </c>
       <c r="C293" s="37" t="s">
         <v>138</v>
@@ -10200,7 +9956,7 @@
         <v>61</v>
       </c>
       <c r="B294" s="31" t="s">
-        <v>365</v>
+        <v>354</v>
       </c>
       <c r="C294" s="37" t="s">
         <v>138</v>
@@ -10212,7 +9968,7 @@
         <v>75</v>
       </c>
       <c r="B295" s="31" t="s">
-        <v>366</v>
+        <v>355</v>
       </c>
       <c r="C295" s="37" t="s">
         <v>138</v>
@@ -10224,7 +9980,7 @@
         <v>75</v>
       </c>
       <c r="B296" s="31" t="s">
-        <v>366</v>
+        <v>355</v>
       </c>
       <c r="C296" s="37" t="s">
         <v>235</v>
@@ -10236,7 +9992,7 @@
         <v>75</v>
       </c>
       <c r="B297" s="31" t="s">
-        <v>367</v>
+        <v>356</v>
       </c>
       <c r="C297" s="37" t="s">
         <v>138</v>
@@ -10248,7 +10004,7 @@
         <v>75</v>
       </c>
       <c r="B298" s="31" t="s">
-        <v>367</v>
+        <v>356</v>
       </c>
       <c r="C298" s="37" t="s">
         <v>235</v>
@@ -10260,7 +10016,7 @@
         <v>75</v>
       </c>
       <c r="B299" s="31" t="s">
-        <v>368</v>
+        <v>357</v>
       </c>
       <c r="C299" s="37" t="s">
         <v>138</v>
@@ -10272,7 +10028,7 @@
         <v>75</v>
       </c>
       <c r="B300" s="31" t="s">
-        <v>368</v>
+        <v>357</v>
       </c>
       <c r="C300" s="37" t="s">
         <v>235</v>
@@ -10284,7 +10040,7 @@
         <v>75</v>
       </c>
       <c r="B301" s="31" t="s">
-        <v>369</v>
+        <v>358</v>
       </c>
       <c r="C301" s="37" t="s">
         <v>138</v>
@@ -10296,7 +10052,7 @@
         <v>75</v>
       </c>
       <c r="B302" s="31" t="s">
-        <v>369</v>
+        <v>358</v>
       </c>
       <c r="C302" s="37" t="s">
         <v>235</v>
@@ -10308,7 +10064,7 @@
         <v>46</v>
       </c>
       <c r="B303" s="31" t="s">
-        <v>370</v>
+        <v>359</v>
       </c>
       <c r="C303" s="37" t="s">
         <v>235</v>
@@ -10320,7 +10076,7 @@
         <v>46</v>
       </c>
       <c r="B304" s="31" t="s">
-        <v>371</v>
+        <v>360</v>
       </c>
       <c r="C304" s="37" t="s">
         <v>138</v>
@@ -10332,7 +10088,7 @@
         <v>62</v>
       </c>
       <c r="B305" s="31" t="s">
-        <v>372</v>
+        <v>361</v>
       </c>
       <c r="C305" s="37" t="s">
         <v>138</v>
@@ -10344,7 +10100,7 @@
         <v>62</v>
       </c>
       <c r="B306" s="31" t="s">
-        <v>373</v>
+        <v>362</v>
       </c>
       <c r="C306" s="37" t="s">
         <v>138</v>
@@ -10356,7 +10112,7 @@
         <v>62</v>
       </c>
       <c r="B307" s="31" t="s">
-        <v>374</v>
+        <v>363</v>
       </c>
       <c r="C307" s="37" t="s">
         <v>138</v>
@@ -10368,7 +10124,7 @@
         <v>69</v>
       </c>
       <c r="B308" s="31" t="s">
-        <v>375</v>
+        <v>364</v>
       </c>
       <c r="C308" s="37" t="s">
         <v>138</v>
@@ -10380,7 +10136,7 @@
         <v>85</v>
       </c>
       <c r="B309" s="31" t="s">
-        <v>376</v>
+        <v>365</v>
       </c>
       <c r="C309" s="37" t="s">
         <v>235</v>
@@ -10392,7 +10148,7 @@
         <v>79</v>
       </c>
       <c r="B310" s="31" t="s">
-        <v>377</v>
+        <v>366</v>
       </c>
       <c r="C310" s="37" t="s">
         <v>138</v>
@@ -10404,7 +10160,7 @@
         <v>79</v>
       </c>
       <c r="B311" s="31" t="s">
-        <v>378</v>
+        <v>367</v>
       </c>
       <c r="C311" s="37" t="s">
         <v>138</v>
@@ -10416,7 +10172,7 @@
         <v>79</v>
       </c>
       <c r="B312" s="31" t="s">
-        <v>379</v>
+        <v>368</v>
       </c>
       <c r="C312" s="37" t="s">
         <v>138</v>
@@ -10428,7 +10184,7 @@
         <v>79</v>
       </c>
       <c r="B313" s="31" t="s">
-        <v>380</v>
+        <v>369</v>
       </c>
       <c r="C313" s="37" t="s">
         <v>138</v>
@@ -10440,7 +10196,7 @@
         <v>79</v>
       </c>
       <c r="B314" s="31" t="s">
-        <v>381</v>
+        <v>370</v>
       </c>
       <c r="C314" s="37" t="s">
         <v>138</v>
@@ -10452,7 +10208,7 @@
         <v>79</v>
       </c>
       <c r="B315" s="31" t="s">
-        <v>382</v>
+        <v>371</v>
       </c>
       <c r="C315" s="37" t="s">
         <v>138</v>
@@ -10464,7 +10220,7 @@
         <v>79</v>
       </c>
       <c r="B316" s="31" t="s">
-        <v>383</v>
+        <v>372</v>
       </c>
       <c r="C316" s="37" t="s">
         <v>138</v>
@@ -10476,7 +10232,7 @@
         <v>79</v>
       </c>
       <c r="B317" s="31" t="s">
-        <v>384</v>
+        <v>373</v>
       </c>
       <c r="C317" s="37" t="s">
         <v>138</v>
@@ -10488,7 +10244,7 @@
         <v>58</v>
       </c>
       <c r="B318" s="31" t="s">
-        <v>385</v>
+        <v>374</v>
       </c>
       <c r="C318" s="37" t="s">
         <v>281</v>
@@ -10500,7 +10256,7 @@
         <v>58</v>
       </c>
       <c r="B319" s="31" t="s">
-        <v>385</v>
+        <v>374</v>
       </c>
       <c r="C319" s="37" t="s">
         <v>138</v>
@@ -10512,7 +10268,7 @@
         <v>58</v>
       </c>
       <c r="B320" s="31" t="s">
-        <v>386</v>
+        <v>375</v>
       </c>
       <c r="C320" s="37" t="s">
         <v>281</v>
@@ -10524,7 +10280,7 @@
         <v>58</v>
       </c>
       <c r="B321" s="31" t="s">
-        <v>387</v>
+        <v>376</v>
       </c>
       <c r="C321" s="37" t="s">
         <v>281</v>
@@ -10536,7 +10292,7 @@
         <v>58</v>
       </c>
       <c r="B322" s="31" t="s">
-        <v>388</v>
+        <v>377</v>
       </c>
       <c r="C322" s="37" t="s">
         <v>281</v>
@@ -10548,7 +10304,7 @@
         <v>58</v>
       </c>
       <c r="B323" s="31" t="s">
-        <v>389</v>
+        <v>378</v>
       </c>
       <c r="C323" s="37" t="s">
         <v>281</v>
@@ -10560,7 +10316,7 @@
         <v>58</v>
       </c>
       <c r="B324" s="31" t="s">
-        <v>389</v>
+        <v>378</v>
       </c>
       <c r="C324" s="37" t="s">
         <v>138</v>
@@ -10572,7 +10328,7 @@
         <v>58</v>
       </c>
       <c r="B325" s="31" t="s">
-        <v>390</v>
+        <v>379</v>
       </c>
       <c r="C325" s="37" t="s">
         <v>281</v>
@@ -10584,7 +10340,7 @@
         <v>58</v>
       </c>
       <c r="B326" s="31" t="s">
-        <v>391</v>
+        <v>380</v>
       </c>
       <c r="C326" s="37" t="s">
         <v>281</v>
@@ -10596,7 +10352,7 @@
         <v>58</v>
       </c>
       <c r="B327" s="31" t="s">
-        <v>392</v>
+        <v>381</v>
       </c>
       <c r="C327" s="37" t="s">
         <v>281</v>
@@ -10608,7 +10364,7 @@
         <v>58</v>
       </c>
       <c r="B328" s="31" t="s">
-        <v>393</v>
+        <v>382</v>
       </c>
       <c r="C328" s="37" t="s">
         <v>281</v>
@@ -10620,7 +10376,7 @@
         <v>58</v>
       </c>
       <c r="B329" s="31" t="s">
-        <v>393</v>
+        <v>382</v>
       </c>
       <c r="C329" s="37" t="s">
         <v>138</v>
@@ -10632,7 +10388,7 @@
         <v>58</v>
       </c>
       <c r="B330" s="31" t="s">
-        <v>394</v>
+        <v>383</v>
       </c>
       <c r="C330" s="37" t="s">
         <v>281</v>
@@ -10644,7 +10400,7 @@
         <v>58</v>
       </c>
       <c r="B331" s="31" t="s">
-        <v>394</v>
+        <v>383</v>
       </c>
       <c r="C331" s="37" t="s">
         <v>138</v>
@@ -10656,7 +10412,7 @@
         <v>58</v>
       </c>
       <c r="B332" s="31" t="s">
-        <v>395</v>
+        <v>384</v>
       </c>
       <c r="C332" s="37" t="s">
         <v>281</v>
@@ -10668,7 +10424,7 @@
         <v>58</v>
       </c>
       <c r="B333" s="31" t="s">
-        <v>396</v>
+        <v>385</v>
       </c>
       <c r="C333" s="37" t="s">
         <v>281</v>
@@ -10680,7 +10436,7 @@
         <v>58</v>
       </c>
       <c r="B334" s="31" t="s">
-        <v>397</v>
+        <v>386</v>
       </c>
       <c r="C334" s="37" t="s">
         <v>281</v>
@@ -10692,7 +10448,7 @@
         <v>58</v>
       </c>
       <c r="B335" s="31" t="s">
-        <v>398</v>
+        <v>387</v>
       </c>
       <c r="C335" s="37" t="s">
         <v>281</v>
@@ -10704,7 +10460,7 @@
         <v>58</v>
       </c>
       <c r="B336" s="31" t="s">
-        <v>399</v>
+        <v>388</v>
       </c>
       <c r="C336" s="37" t="s">
         <v>281</v>
@@ -10716,7 +10472,7 @@
         <v>58</v>
       </c>
       <c r="B337" s="31" t="s">
-        <v>400</v>
+        <v>389</v>
       </c>
       <c r="C337" s="37" t="s">
         <v>281</v>
@@ -10752,7 +10508,7 @@
         <v>67</v>
       </c>
       <c r="B340" s="31" t="s">
-        <v>401</v>
+        <v>390</v>
       </c>
       <c r="C340" s="37" t="s">
         <v>138</v>
@@ -10764,7 +10520,7 @@
         <v>67</v>
       </c>
       <c r="B341" s="31" t="s">
-        <v>402</v>
+        <v>391</v>
       </c>
       <c r="C341" s="37" t="s">
         <v>235</v>
@@ -10776,7 +10532,7 @@
         <v>67</v>
       </c>
       <c r="B342" s="31" t="s">
-        <v>403</v>
+        <v>392</v>
       </c>
       <c r="C342" s="37" t="s">
         <v>235</v>
@@ -10788,7 +10544,7 @@
         <v>67</v>
       </c>
       <c r="B343" s="31" t="s">
-        <v>404</v>
+        <v>393</v>
       </c>
       <c r="C343" s="37" t="s">
         <v>138</v>
@@ -10800,7 +10556,7 @@
         <v>67</v>
       </c>
       <c r="B344" s="31" t="s">
-        <v>404</v>
+        <v>393</v>
       </c>
       <c r="C344" s="37" t="s">
         <v>235</v>
@@ -10812,7 +10568,7 @@
         <v>67</v>
       </c>
       <c r="B345" s="31" t="s">
-        <v>405</v>
+        <v>394</v>
       </c>
       <c r="C345" s="37" t="s">
         <v>281</v>
@@ -10824,7 +10580,7 @@
         <v>67</v>
       </c>
       <c r="B346" s="31" t="s">
-        <v>405</v>
+        <v>394</v>
       </c>
       <c r="C346" s="37" t="s">
         <v>138</v>
@@ -11252,12 +11008,12 @@
       <c r="D416" s="34"/>
     </row>
     <row r="417" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A417" s="45" t="s">
+      <c r="A417" s="48" t="s">
         <v>95</v>
       </c>
-      <c r="B417" s="42"/>
-      <c r="C417" s="42"/>
-      <c r="D417" s="42"/>
+      <c r="B417" s="45"/>
+      <c r="C417" s="45"/>
+      <c r="D417" s="45"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -11295,11 +11051,11 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" ht="28" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="44" t="s">
+      <c r="A1" s="47" t="s">
         <v>96</v>
       </c>
-      <c r="B1" s="42"/>
-      <c r="C1" s="42"/>
+      <c r="B1" s="45"/>
+      <c r="C1" s="45"/>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2" s="3" t="s">
@@ -11375,7 +11131,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
-  <dimension ref="A1:B31"/>
+  <dimension ref="A1:B32"/>
   <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
@@ -11383,10 +11139,10 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2" ht="28" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="44" t="s">
+      <c r="A1" s="47" t="s">
         <v>102</v>
       </c>
-      <c r="B1" s="42"/>
+      <c r="B1" s="45"/>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A2" s="3" t="s">
@@ -11615,7 +11371,7 @@
       </c>
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A30" s="47" t="s">
+      <c r="A30" s="42" t="s">
         <v>250</v>
       </c>
       <c r="B30" s="26">
@@ -11624,12 +11380,21 @@
       </c>
     </row>
     <row r="31" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A31" s="40" t="s">
-        <v>292</v>
-      </c>
-      <c r="B31" s="24">
+      <c r="A31" s="42" t="s">
+        <v>287</v>
+      </c>
+      <c r="B31" s="26">
         <f>SUM('📈 HISTÓRICO CONSEJOS'!B31:T31)</f>
         <v>73825</v>
+      </c>
+    </row>
+    <row r="32" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A32" s="40" t="s">
+        <v>395</v>
+      </c>
+      <c r="B32" s="24">
+        <f>SUM('📈 HISTÓRICO CONSEJOS'!B32:T32)</f>
+        <v>1392</v>
       </c>
     </row>
   </sheetData>
@@ -11643,7 +11408,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
-  <dimension ref="A1:T31"/>
+  <dimension ref="A1:T32"/>
   <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="16" customWidth="1"/>
@@ -11651,28 +11416,28 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:20" ht="28" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="44" t="s">
+      <c r="A1" s="47" t="s">
         <v>128</v>
       </c>
-      <c r="B1" s="42"/>
-      <c r="C1" s="42"/>
-      <c r="D1" s="42"/>
-      <c r="E1" s="42"/>
-      <c r="F1" s="42"/>
-      <c r="G1" s="42"/>
-      <c r="H1" s="42"/>
-      <c r="I1" s="42"/>
-      <c r="J1" s="42"/>
-      <c r="K1" s="42"/>
-      <c r="L1" s="42"/>
-      <c r="M1" s="42"/>
-      <c r="N1" s="42"/>
-      <c r="O1" s="42"/>
-      <c r="P1" s="42"/>
-      <c r="Q1" s="42"/>
-      <c r="R1" s="42"/>
-      <c r="S1" s="42"/>
-      <c r="T1" s="42"/>
+      <c r="B1" s="45"/>
+      <c r="C1" s="45"/>
+      <c r="D1" s="45"/>
+      <c r="E1" s="45"/>
+      <c r="F1" s="45"/>
+      <c r="G1" s="45"/>
+      <c r="H1" s="45"/>
+      <c r="I1" s="45"/>
+      <c r="J1" s="45"/>
+      <c r="K1" s="45"/>
+      <c r="L1" s="45"/>
+      <c r="M1" s="45"/>
+      <c r="N1" s="45"/>
+      <c r="O1" s="45"/>
+      <c r="P1" s="45"/>
+      <c r="Q1" s="45"/>
+      <c r="R1" s="45"/>
+      <c r="S1" s="45"/>
+      <c r="T1" s="45"/>
     </row>
     <row r="2" spans="1:20" ht="39" x14ac:dyDescent="0.35">
       <c r="A2" s="3" t="s">
@@ -13411,7 +13176,7 @@
       </c>
     </row>
     <row r="30" spans="1:20" s="20" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A30" s="48" t="s">
+      <c r="A30" s="43" t="s">
         <v>250</v>
       </c>
       <c r="B30" s="11">
@@ -13472,67 +13237,97 @@
         <v>22893</v>
       </c>
     </row>
-    <row r="31" spans="1:20" s="33" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A31" s="39" t="s">
+    <row r="31" spans="1:20" s="20" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A31" s="43" t="s">
         <v>287</v>
       </c>
-      <c r="B31" s="5">
+      <c r="B31" s="11">
         <v>719</v>
       </c>
-      <c r="C31" s="5">
+      <c r="C31" s="11">
         <v>232</v>
       </c>
-      <c r="D31" s="13">
+      <c r="D31" s="11">
         <v>441</v>
       </c>
-      <c r="E31" s="5">
+      <c r="E31" s="11">
         <v>279</v>
       </c>
-      <c r="F31" s="5">
+      <c r="F31" s="11">
         <v>231</v>
       </c>
-      <c r="G31" s="5">
+      <c r="G31" s="11">
         <v>1985</v>
       </c>
-      <c r="H31" s="5">
+      <c r="H31" s="11">
         <v>1377</v>
       </c>
-      <c r="I31" s="5">
+      <c r="I31" s="11">
         <v>4640</v>
       </c>
-      <c r="J31" s="5">
+      <c r="J31" s="11">
         <v>23</v>
       </c>
-      <c r="K31" s="5">
+      <c r="K31" s="11">
         <v>3074</v>
       </c>
-      <c r="L31" s="5">
+      <c r="L31" s="11">
         <v>4356</v>
       </c>
-      <c r="M31" s="5">
+      <c r="M31" s="11">
         <v>426</v>
       </c>
-      <c r="N31" s="5">
+      <c r="N31" s="11">
         <v>336</v>
       </c>
-      <c r="O31" s="5">
+      <c r="O31" s="11">
         <v>15059</v>
       </c>
-      <c r="P31" s="5">
+      <c r="P31" s="11">
         <v>7385</v>
       </c>
-      <c r="Q31" s="5">
+      <c r="Q31" s="11">
         <v>9274</v>
       </c>
-      <c r="R31" s="5">
+      <c r="R31" s="11">
         <v>500</v>
       </c>
-      <c r="S31" s="5">
+      <c r="S31" s="11">
         <v>309</v>
       </c>
-      <c r="T31" s="5">
+      <c r="T31" s="11">
         <v>23179</v>
       </c>
+    </row>
+    <row r="32" spans="1:20" s="33" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A32" s="39" t="s">
+        <v>395</v>
+      </c>
+      <c r="B32" s="5">
+        <v>719</v>
+      </c>
+      <c r="C32" s="5">
+        <v>232</v>
+      </c>
+      <c r="D32" s="13">
+        <v>441</v>
+      </c>
+      <c r="E32" s="5"/>
+      <c r="F32" s="5"/>
+      <c r="G32" s="5"/>
+      <c r="H32" s="5"/>
+      <c r="I32" s="5"/>
+      <c r="J32" s="5"/>
+      <c r="K32" s="5"/>
+      <c r="L32" s="5"/>
+      <c r="M32" s="5"/>
+      <c r="N32" s="5"/>
+      <c r="O32" s="5"/>
+      <c r="P32" s="5"/>
+      <c r="Q32" s="5"/>
+      <c r="R32" s="5"/>
+      <c r="S32" s="5"/>
+      <c r="T32" s="5"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>